<commit_message>
Remove WP Engine from the published market screen
</commit_message>
<xml_diff>
--- a/assets/documents/wordpress-job-market-screen-live-states.xlsx
+++ b/assets/documents/wordpress-job-market-screen-live-states.xlsx
@@ -6,14 +6,14 @@
     <sheet state="visible" name="Live States" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Live States'!$A$1:$G$11</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Live States'!$A$1:$G$10</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="54">
   <si>
     <t>Job title</t>
   </si>
@@ -175,15 +175,6 @@
   </si>
   <si>
     <t>Q2 fails: WordPress is optional rather than the operational center of the role.</t>
-  </si>
-  <si>
-    <t>Technical Support L1</t>
-  </si>
-  <si>
-    <t>WP Engine</t>
-  </si>
-  <si>
-    <t>Q1–Q3 pass: WordPress, DNS, Linux command-line, and customer troubleshooting work.</t>
   </si>
 </sst>
 </file>
@@ -771,31 +762,8 @@
         <v>53</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="G11" s="12" t="s">
-        <v>56</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="$A$1:$G$11"/>
+  <autoFilter ref="$A$1:$G$10"/>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
     <hyperlink r:id="rId2" ref="C3"/>

</xml_diff>